<commit_message>
Fixed font security issues
</commit_message>
<xml_diff>
--- a/apps/docs-firefly/release-schedule.xlsx
+++ b/apps/docs-firefly/release-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andredavcev/Projects/theory/apps/docs-firefly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872F0787-D049-034B-8DC8-990C387897E2}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{855573FB-B4C5-3E47-B20A-883A5771FEF8}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
+    <workbookView xWindow="1500" yWindow="560" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
   <si>
     <t>Version</t>
   </si>
@@ -217,6 +217,9 @@
   </si>
   <si>
     <t>JIRA Workflows</t>
+  </si>
+  <si>
+    <t>Find Event Now Firefly Button</t>
   </si>
 </sst>
 </file>
@@ -578,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E808F83-7B39-7A4C-8F08-E0AB4C8C7AD2}">
-  <dimension ref="B2:E43"/>
+  <dimension ref="B2:E44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -793,87 +796,92 @@
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>19</v>
-      </c>
-      <c r="C34" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D35" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C41" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C42" t="s">
-        <v>54</v>
-      </c>
-      <c r="D42" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
+        <v>55</v>
+      </c>
+      <c r="C43" t="s">
+        <v>54</v>
+      </c>
+      <c r="D43" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
         <v>57</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C44" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added vs code extension "github.vscode-pull-request-github"
</commit_message>
<xml_diff>
--- a/apps/docs-firefly/release-schedule.xlsx
+++ b/apps/docs-firefly/release-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andredavcev/Projects/theory/apps/docs-firefly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{855573FB-B4C5-3E47-B20A-883A5771FEF8}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E203EFB3-9CAB-0F4E-A36D-919C542A3961}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1500" yWindow="560" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
   <si>
     <t>Version</t>
   </si>
@@ -220,6 +220,12 @@
   </si>
   <si>
     <t>Find Event Now Firefly Button</t>
+  </si>
+  <si>
+    <t>Jest Testing</t>
+  </si>
+  <si>
+    <t>Custom Notification Background Colors</t>
   </si>
 </sst>
 </file>
@@ -581,11 +587,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E808F83-7B39-7A4C-8F08-E0AB4C8C7AD2}">
-  <dimension ref="B2:E44"/>
+  <dimension ref="B2:E46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.83203125" bestFit="1" customWidth="1"/>
@@ -762,126 +768,136 @@
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>50</v>
+        <v>17</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>64</v>
+        <v>18</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>19</v>
-      </c>
-      <c r="C35" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>20</v>
-      </c>
-      <c r="C36" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="D37" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C38" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C39" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C40" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C41" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="C42" t="s">
-        <v>53</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="C43" t="s">
-        <v>54</v>
-      </c>
-      <c r="D43" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" t="s">
+        <v>54</v>
+      </c>
+      <c r="D45" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
         <v>57</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C46" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tiny commit for .gitignore
</commit_message>
<xml_diff>
--- a/apps/docs-firefly/release-schedule.xlsx
+++ b/apps/docs-firefly/release-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andredavcev/Projects/theory/apps/docs-firefly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E203EFB3-9CAB-0F4E-A36D-919C542A3961}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1236B4-4AB0-3042-868E-4CF50799DD12}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1500" yWindow="560" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
   <si>
     <t>Version</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>Custom Notification Background Colors</t>
+  </si>
+  <si>
+    <t>Auth</t>
   </si>
 </sst>
 </file>
@@ -587,7 +590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E808F83-7B39-7A4C-8F08-E0AB4C8C7AD2}">
-  <dimension ref="B2:E46"/>
+  <dimension ref="B2:E47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -671,233 +674,238 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C12" t="s">
-        <v>6</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>30</v>
+        <v>58</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>27</v>
+        <v>45</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="D22" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>50</v>
+        <v>17</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>18</v>
-      </c>
-      <c r="C34" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>64</v>
+        <v>18</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>19</v>
-      </c>
-      <c r="C37" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D38" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C45" t="s">
-        <v>54</v>
-      </c>
-      <c r="D45" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46" t="s">
+        <v>54</v>
+      </c>
+      <c r="D46" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B47" t="s">
         <v>57</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>